<commit_message>
new report with the count of vessels inside hormuz, and it's distribution
</commit_message>
<xml_diff>
--- a/afra_scale_mapping.xlsx
+++ b/afra_scale_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jainglobalcom-my.sharepoint.com/personal/luiscarlos_gaitan_jainglobal_com/Documents/Coding/vessel_crossing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{C2E60958-AAAA-47D2-BF2D-015761F03F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E60A30FB-18AD-431C-8245-090452DADC89}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{C2E60958-AAAA-47D2-BF2D-015761F03F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EDB8BB9-9799-43E3-A525-7B6D0B9A8C39}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="29010" windowHeight="23385" xr2:uid="{A4DC2974-25D8-4ECA-9D90-52E65D1B1760}"/>
+    <workbookView xWindow="3285" yWindow="3285" windowWidth="43200" windowHeight="17145" xr2:uid="{A4DC2974-25D8-4ECA-9D90-52E65D1B1760}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -157,6 +157,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -481,8 +485,8 @@
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>